<commit_message>
Optimisation de l'interface utilisateur
</commit_message>
<xml_diff>
--- a/data/excelphase2.xlsx
+++ b/data/excelphase2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\owner\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\owner\Documents\Excelium\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{880B519C-BFEB-4430-8E3B-127C0DB4D931}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{224CE5A7-CFF3-4A2F-813D-C0B7A457BC2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1598" yWindow="698" windowWidth="16200" windowHeight="9307" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2948" yWindow="2048" windowWidth="16200" windowHeight="9307" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Etudiants" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="102">
   <si>
     <t>Nom</t>
   </si>
@@ -365,8 +365,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1230,7 +1231,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.45">
@@ -1371,6 +1372,20 @@
       </c>
       <c r="F7" t="s">
         <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>71</v>
+      </c>
+      <c r="B8" s="1">
+        <v>0.375</v>
+      </c>
+      <c r="C8" s="1">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="D8" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ignorer les feuilles Excel vides à l'import
</commit_message>
<xml_diff>
--- a/data/excelphase2.xlsx
+++ b/data/excelphase2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\owner\Documents\Excelium\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{224CE5A7-CFF3-4A2F-813D-C0B7A457BC2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1DE4EB9-6A16-4849-80BE-9E59D46B316E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2948" yWindow="2048" windowWidth="16200" windowHeight="9307" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2948" yWindow="2048" windowWidth="16200" windowHeight="9307" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Etudiants" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="87">
   <si>
     <t>Nom</t>
   </si>
@@ -173,52 +173,7 @@
     <t>Luc Moreau</t>
   </si>
   <si>
-    <t>Anciennete</t>
-  </si>
-  <si>
-    <t>Bureau</t>
-  </si>
-  <si>
-    <t>Courriel</t>
-  </si>
-  <si>
-    <t>ChargeCours</t>
-  </si>
-  <si>
-    <t>A-210</t>
-  </si>
-  <si>
-    <t>jean@udem.ca</t>
-  </si>
-  <si>
-    <t>A-214</t>
-  </si>
-  <si>
-    <t>sophie@udem.ca</t>
-  </si>
-  <si>
     <t>A-110</t>
-  </si>
-  <si>
-    <t>marc@udem.ca</t>
-  </si>
-  <si>
-    <t>A-305</t>
-  </si>
-  <si>
-    <t>julie@udem.ca</t>
-  </si>
-  <si>
-    <t>B-210</t>
-  </si>
-  <si>
-    <t>paul@udem.ca</t>
-  </si>
-  <si>
-    <t>B-320</t>
-  </si>
-  <si>
-    <t>claire@udem.ca</t>
   </si>
   <si>
     <t>Jour</t>
@@ -698,7 +653,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
@@ -721,7 +676,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
@@ -744,7 +699,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="B4" t="s">
         <v>13</v>
@@ -767,7 +722,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="B5" t="s">
         <v>15</v>
@@ -790,7 +745,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="B6" t="s">
         <v>7</v>
@@ -813,7 +768,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="B7" t="s">
         <v>18</v>
@@ -836,7 +791,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="B8" t="s">
         <v>19</v>
@@ -859,7 +814,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="B9" t="s">
         <v>7</v>
@@ -1081,150 +1036,9 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D1" t="s">
-        <v>50</v>
-      </c>
-      <c r="E1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C2">
-        <v>12</v>
-      </c>
-      <c r="D2" t="s">
-        <v>53</v>
-      </c>
-      <c r="E2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C3">
-        <v>8</v>
-      </c>
-      <c r="D3" t="s">
-        <v>55</v>
-      </c>
-      <c r="E3" t="s">
-        <v>56</v>
-      </c>
-      <c r="F3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C4">
-        <v>15</v>
-      </c>
-      <c r="D4" t="s">
-        <v>57</v>
-      </c>
-      <c r="E4" t="s">
-        <v>58</v>
-      </c>
-      <c r="F4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B5" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5">
-        <v>5</v>
-      </c>
-      <c r="D5" t="s">
-        <v>59</v>
-      </c>
-      <c r="E5" t="s">
-        <v>60</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
-        <v>42</v>
-      </c>
-      <c r="B6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C6">
-        <v>20</v>
-      </c>
-      <c r="D6" t="s">
-        <v>61</v>
-      </c>
-      <c r="E6" t="s">
-        <v>62</v>
-      </c>
-      <c r="F6">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>45</v>
-      </c>
-      <c r="B7" t="s">
-        <v>41</v>
-      </c>
-      <c r="C7">
-        <v>10</v>
-      </c>
-      <c r="D7" t="s">
-        <v>63</v>
-      </c>
-      <c r="E7" t="s">
-        <v>64</v>
-      </c>
-      <c r="F7">
-        <v>3</v>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1236,79 +1050,79 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="B1" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="C1" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="D1" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="E1" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="F1" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="B2" t="s">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="C2" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="D2" t="s">
         <v>26</v>
       </c>
       <c r="E2" t="s">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="F2" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="B3" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="C3" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="D3" t="s">
         <v>30</v>
       </c>
       <c r="E3" t="s">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="F3" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>79</v>
+        <v>64</v>
       </c>
       <c r="B4" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="C4" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="D4" t="s">
         <v>39</v>
       </c>
       <c r="E4" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="F4" t="s">
         <v>9</v>
@@ -1316,59 +1130,59 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="B5" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="C5" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="D5" t="s">
         <v>36</v>
       </c>
       <c r="E5" t="s">
-        <v>83</v>
+        <v>68</v>
       </c>
       <c r="F5" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
       <c r="B6" t="s">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="C6" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="D6" t="s">
         <v>33</v>
       </c>
       <c r="E6" t="s">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="F6" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="B7" t="s">
-        <v>87</v>
+        <v>72</v>
       </c>
       <c r="C7" t="s">
-        <v>88</v>
+        <v>73</v>
       </c>
       <c r="D7" t="s">
         <v>46</v>
       </c>
       <c r="E7" t="s">
-        <v>89</v>
+        <v>74</v>
       </c>
       <c r="F7" t="s">
         <v>9</v>
@@ -1376,7 +1190,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="B8" s="1">
         <v>0.375</v>
@@ -1403,16 +1217,16 @@
         <v>2</v>
       </c>
       <c r="B1" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="C1" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="D1" t="s">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="E1" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
@@ -1420,7 +1234,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="B2" t="s">
         <v>26</v>
@@ -1440,7 +1254,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="B3" t="s">
         <v>30</v>
@@ -1460,7 +1274,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="B4" t="s">
         <v>33</v>
@@ -1480,7 +1294,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="B5" t="s">
         <v>39</v>
@@ -1500,7 +1314,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="B6" t="s">
         <v>43</v>
@@ -1520,7 +1334,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="B7" t="s">
         <v>46</v>

</xml_diff>